<commit_message>
feat: harden final package and format validation
</commit_message>
<xml_diff>
--- a/skills/build-k12-research-project/assets/templates/project-data-workbook.xlsx
+++ b/skills/build-k12-research-project/assets/templates/project-data-workbook.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目说明" sheetId="1" r:id="R47eb18b2daff4fd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变量编码" sheetId="2" r:id="R8ba3d05edccc4895"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原始数据" sheetId="3" r:id="R0ab339241d9b472d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="清理编码" sheetId="4" r:id="R266f3a57bc124791"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计分析" sheetId="5" r:id="R0ba098d07a634248"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图表结果" sheetId="6" r:id="R48c978c8373f4baa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据索引" sheetId="7" r:id="R427dbe825c1f49ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="照片登记" sheetId="8" r:id="R0423c47202ee4879"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材料进度" sheetId="9" r:id="Rd02c1008a0a74bb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目说明" sheetId="1" r:id="R195a206a49194776"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变量编码" sheetId="2" r:id="Re9b2890cbcf046c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原始数据" sheetId="3" r:id="R563a50393b6641b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="清理编码" sheetId="4" r:id="R9bf850bf872a43f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计分析" sheetId="5" r:id="R6795338bd8704ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图表结果" sheetId="6" r:id="Rf9f8885d820c425c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据索引" sheetId="7" r:id="R60e4d165f140438d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="照片登记" sheetId="8" r:id="Rf4dd6d8a5b914526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材料进度" sheetId="9" r:id="Rc38805780d654072"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -238,27 +238,31 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="EvidenceIndex" displayName="EvidenceIndex" ref="A3:K33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="11">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="EvidenceIndex" displayName="EvidenceIndex" ref="A3:O33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="15">
     <x:tableColumn id="1" name="证据ID"/>
     <x:tableColumn id="2" name="类型"/>
     <x:tableColumn id="3" name="真实日期"/>
-    <x:tableColumn id="4" name="相对文件路径"/>
-    <x:tableColumn id="5" name="SHA-256"/>
-    <x:tableColumn id="6" name="对应问题"/>
-    <x:tableColumn id="7" name="对应材料"/>
-    <x:tableColumn id="8" name="对应结论"/>
-    <x:tableColumn id="9" name="隐私等级"/>
-    <x:tableColumn id="10" name="授权/核验状态"/>
-    <x:tableColumn id="11" name="责任人"/>
+    <x:tableColumn id="4" name="是否随包"/>
+    <x:tableColumn id="5" name="交付相对路径"/>
+    <x:tableColumn id="6" name="SHA-256"/>
+    <x:tableColumn id="7" name="保管责任人"/>
+    <x:tableColumn id="8" name="受控定位"/>
+    <x:tableColumn id="9" name="保管核验日期"/>
+    <x:tableColumn id="10" name="对应问题"/>
+    <x:tableColumn id="11" name="对应材料"/>
+    <x:tableColumn id="12" name="对应结论"/>
+    <x:tableColumn id="13" name="隐私等级"/>
+    <x:tableColumn id="14" name="授权/核验状态"/>
+    <x:tableColumn id="15" name="责任人"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PhotoRegister" displayName="PhotoRegister" ref="A3:O33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="15">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PhotoRegister" displayName="PhotoRegister" ref="A3:T33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="20">
     <x:tableColumn id="1" name="照片ID"/>
     <x:tableColumn id="2" name="原文件名"/>
     <x:tableColumn id="3" name="原件SHA-256"/>
@@ -266,14 +270,19 @@
     <x:tableColumn id="5" name="地点"/>
     <x:tableColumn id="6" name="活动"/>
     <x:tableColumn id="7" name="拍摄/来源"/>
-    <x:tableColumn id="8" name="授权状态"/>
-    <x:tableColumn id="9" name="人物处理"/>
-    <x:tableColumn id="10" name="图题"/>
-    <x:tableColumn id="11" name="替代文本"/>
-    <x:tableColumn id="12" name="对应材料/案例"/>
-    <x:tableColumn id="13" name="派生文件"/>
-    <x:tableColumn id="14" name="派生SHA-256"/>
-    <x:tableColumn id="15" name="图号/位置"/>
+    <x:tableColumn id="8" name="是否随包"/>
+    <x:tableColumn id="9" name="原件相对路径"/>
+    <x:tableColumn id="10" name="保管责任人"/>
+    <x:tableColumn id="11" name="受控定位"/>
+    <x:tableColumn id="12" name="保管核验日期"/>
+    <x:tableColumn id="13" name="授权状态"/>
+    <x:tableColumn id="14" name="人物处理"/>
+    <x:tableColumn id="15" name="图题"/>
+    <x:tableColumn id="16" name="替代文本"/>
+    <x:tableColumn id="17" name="对应材料/案例"/>
+    <x:tableColumn id="18" name="派生文件"/>
+    <x:tableColumn id="19" name="派生SHA-256"/>
+    <x:tableColumn id="20" name="图号/位置"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -493,7 +502,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
@@ -900,13 +909,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf305028724934c95"/>
+    <x:tablePart ns1:id="R6c73998b7fd64ac6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
@@ -1406,13 +1415,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab818de6166e4dee"/>
+    <x:tablePart ns1:id="R002b8f914dfb4d31"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
@@ -1798,13 +1807,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53a0b82da05f4a69"/>
+    <x:tablePart ns1:id="R321e30dea1cb42b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
@@ -2634,13 +2643,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94431a5cc9694560"/>
+    <x:tablePart ns1:id="R598c888a9cb942bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
@@ -3027,13 +3036,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74daab6d867244c3"/>
+    <x:tablePart ns1:id="R17c5bcab446841ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
@@ -3541,526 +3550,35 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54ff1d7fcf40403d"/>
+    <x:tablePart ns1:id="R9e098c39c3e44643"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="36" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="68" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="36" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="68" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="30" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="2" t="str">
         <x:v>证据索引</x:v>
-      </x:c>
-      <x:c r="B1" s="2"/>
-      <x:c r="C1" s="2"/>
-      <x:c r="D1" s="2"/>
-      <x:c r="E1" s="2"/>
-      <x:c r="F1" s="2"/>
-      <x:c r="G1" s="2"/>
-      <x:c r="H1" s="2"/>
-      <x:c r="I1" s="2"/>
-      <x:c r="J1" s="2"/>
-      <x:c r="K1" s="2"/>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="5" t="str">
-        <x:v>每条结论链接到真实原件；文件路径优先使用材料包内相对路径。</x:v>
-      </x:c>
-      <x:c r="B2" s="5"/>
-      <x:c r="C2" s="5"/>
-      <x:c r="D2" s="5"/>
-      <x:c r="E2" s="5"/>
-      <x:c r="F2" s="5"/>
-      <x:c r="G2" s="5"/>
-      <x:c r="H2" s="5"/>
-      <x:c r="I2" s="5"/>
-      <x:c r="J2" s="5"/>
-      <x:c r="K2" s="5"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="10" t="str">
-        <x:v>证据ID</x:v>
-      </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>类型</x:v>
-      </x:c>
-      <x:c r="C3" s="10" t="str">
-        <x:v>真实日期</x:v>
-      </x:c>
-      <x:c r="D3" s="10" t="str">
-        <x:v>相对文件路径</x:v>
-      </x:c>
-      <x:c r="E3" s="10" t="str">
-        <x:v>SHA-256</x:v>
-      </x:c>
-      <x:c r="F3" s="10" t="str">
-        <x:v>对应问题</x:v>
-      </x:c>
-      <x:c r="G3" s="10" t="str">
-        <x:v>对应材料</x:v>
-      </x:c>
-      <x:c r="H3" s="10" t="str">
-        <x:v>对应结论</x:v>
-      </x:c>
-      <x:c r="I3" s="10" t="str">
-        <x:v>隐私等级</x:v>
-      </x:c>
-      <x:c r="J3" s="10" t="str">
-        <x:v>授权/核验状态</x:v>
-      </x:c>
-      <x:c r="K3" s="10" t="str">
-        <x:v>责任人</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="14"/>
-      <x:c r="B4" s="14"/>
-      <x:c r="C4" s="15"/>
-      <x:c r="D4" s="14"/>
-      <x:c r="E4" s="14"/>
-      <x:c r="F4" s="14"/>
-      <x:c r="G4" s="14"/>
-      <x:c r="H4" s="14"/>
-      <x:c r="I4" s="14"/>
-      <x:c r="J4" s="14"/>
-      <x:c r="K4" s="14"/>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="14"/>
-      <x:c r="B5" s="14"/>
-      <x:c r="C5" s="15"/>
-      <x:c r="D5" s="14"/>
-      <x:c r="E5" s="14"/>
-      <x:c r="F5" s="14"/>
-      <x:c r="G5" s="14"/>
-      <x:c r="H5" s="14"/>
-      <x:c r="I5" s="14"/>
-      <x:c r="J5" s="14"/>
-      <x:c r="K5" s="14"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="14"/>
-      <x:c r="B6" s="14"/>
-      <x:c r="C6" s="15"/>
-      <x:c r="D6" s="14"/>
-      <x:c r="E6" s="14"/>
-      <x:c r="F6" s="14"/>
-      <x:c r="G6" s="14"/>
-      <x:c r="H6" s="14"/>
-      <x:c r="I6" s="14"/>
-      <x:c r="J6" s="14"/>
-      <x:c r="K6" s="14"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="14"/>
-      <x:c r="B7" s="14"/>
-      <x:c r="C7" s="15"/>
-      <x:c r="D7" s="14"/>
-      <x:c r="E7" s="14"/>
-      <x:c r="F7" s="14"/>
-      <x:c r="G7" s="14"/>
-      <x:c r="H7" s="14"/>
-      <x:c r="I7" s="14"/>
-      <x:c r="J7" s="14"/>
-      <x:c r="K7" s="14"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="14"/>
-      <x:c r="B8" s="14"/>
-      <x:c r="C8" s="15"/>
-      <x:c r="D8" s="14"/>
-      <x:c r="E8" s="14"/>
-      <x:c r="F8" s="14"/>
-      <x:c r="G8" s="14"/>
-      <x:c r="H8" s="14"/>
-      <x:c r="I8" s="14"/>
-      <x:c r="J8" s="14"/>
-      <x:c r="K8" s="14"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="14"/>
-      <x:c r="B9" s="14"/>
-      <x:c r="C9" s="15"/>
-      <x:c r="D9" s="14"/>
-      <x:c r="E9" s="14"/>
-      <x:c r="F9" s="14"/>
-      <x:c r="G9" s="14"/>
-      <x:c r="H9" s="14"/>
-      <x:c r="I9" s="14"/>
-      <x:c r="J9" s="14"/>
-      <x:c r="K9" s="14"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="14"/>
-      <x:c r="B10" s="14"/>
-      <x:c r="C10" s="15"/>
-      <x:c r="D10" s="14"/>
-      <x:c r="E10" s="14"/>
-      <x:c r="F10" s="14"/>
-      <x:c r="G10" s="14"/>
-      <x:c r="H10" s="14"/>
-      <x:c r="I10" s="14"/>
-      <x:c r="J10" s="14"/>
-      <x:c r="K10" s="14"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="14"/>
-      <x:c r="B11" s="14"/>
-      <x:c r="C11" s="15"/>
-      <x:c r="D11" s="14"/>
-      <x:c r="E11" s="14"/>
-      <x:c r="F11" s="14"/>
-      <x:c r="G11" s="14"/>
-      <x:c r="H11" s="14"/>
-      <x:c r="I11" s="14"/>
-      <x:c r="J11" s="14"/>
-      <x:c r="K11" s="14"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="14"/>
-      <x:c r="B12" s="14"/>
-      <x:c r="C12" s="15"/>
-      <x:c r="D12" s="14"/>
-      <x:c r="E12" s="14"/>
-      <x:c r="F12" s="14"/>
-      <x:c r="G12" s="14"/>
-      <x:c r="H12" s="14"/>
-      <x:c r="I12" s="14"/>
-      <x:c r="J12" s="14"/>
-      <x:c r="K12" s="14"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="14"/>
-      <x:c r="B13" s="14"/>
-      <x:c r="C13" s="15"/>
-      <x:c r="D13" s="14"/>
-      <x:c r="E13" s="14"/>
-      <x:c r="F13" s="14"/>
-      <x:c r="G13" s="14"/>
-      <x:c r="H13" s="14"/>
-      <x:c r="I13" s="14"/>
-      <x:c r="J13" s="14"/>
-      <x:c r="K13" s="14"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="14"/>
-      <x:c r="B14" s="14"/>
-      <x:c r="C14" s="15"/>
-      <x:c r="D14" s="14"/>
-      <x:c r="E14" s="14"/>
-      <x:c r="F14" s="14"/>
-      <x:c r="G14" s="14"/>
-      <x:c r="H14" s="14"/>
-      <x:c r="I14" s="14"/>
-      <x:c r="J14" s="14"/>
-      <x:c r="K14" s="14"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="14"/>
-      <x:c r="B15" s="14"/>
-      <x:c r="C15" s="15"/>
-      <x:c r="D15" s="14"/>
-      <x:c r="E15" s="14"/>
-      <x:c r="F15" s="14"/>
-      <x:c r="G15" s="14"/>
-      <x:c r="H15" s="14"/>
-      <x:c r="I15" s="14"/>
-      <x:c r="J15" s="14"/>
-      <x:c r="K15" s="14"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="14"/>
-      <x:c r="B16" s="14"/>
-      <x:c r="C16" s="15"/>
-      <x:c r="D16" s="14"/>
-      <x:c r="E16" s="14"/>
-      <x:c r="F16" s="14"/>
-      <x:c r="G16" s="14"/>
-      <x:c r="H16" s="14"/>
-      <x:c r="I16" s="14"/>
-      <x:c r="J16" s="14"/>
-      <x:c r="K16" s="14"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="14"/>
-      <x:c r="B17" s="14"/>
-      <x:c r="C17" s="15"/>
-      <x:c r="D17" s="14"/>
-      <x:c r="E17" s="14"/>
-      <x:c r="F17" s="14"/>
-      <x:c r="G17" s="14"/>
-      <x:c r="H17" s="14"/>
-      <x:c r="I17" s="14"/>
-      <x:c r="J17" s="14"/>
-      <x:c r="K17" s="14"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="14"/>
-      <x:c r="B18" s="14"/>
-      <x:c r="C18" s="15"/>
-      <x:c r="D18" s="14"/>
-      <x:c r="E18" s="14"/>
-      <x:c r="F18" s="14"/>
-      <x:c r="G18" s="14"/>
-      <x:c r="H18" s="14"/>
-      <x:c r="I18" s="14"/>
-      <x:c r="J18" s="14"/>
-      <x:c r="K18" s="14"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="14"/>
-      <x:c r="B19" s="14"/>
-      <x:c r="C19" s="15"/>
-      <x:c r="D19" s="14"/>
-      <x:c r="E19" s="14"/>
-      <x:c r="F19" s="14"/>
-      <x:c r="G19" s="14"/>
-      <x:c r="H19" s="14"/>
-      <x:c r="I19" s="14"/>
-      <x:c r="J19" s="14"/>
-      <x:c r="K19" s="14"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="14"/>
-      <x:c r="B20" s="14"/>
-      <x:c r="C20" s="15"/>
-      <x:c r="D20" s="14"/>
-      <x:c r="E20" s="14"/>
-      <x:c r="F20" s="14"/>
-      <x:c r="G20" s="14"/>
-      <x:c r="H20" s="14"/>
-      <x:c r="I20" s="14"/>
-      <x:c r="J20" s="14"/>
-      <x:c r="K20" s="14"/>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="14"/>
-      <x:c r="B21" s="14"/>
-      <x:c r="C21" s="15"/>
-      <x:c r="D21" s="14"/>
-      <x:c r="E21" s="14"/>
-      <x:c r="F21" s="14"/>
-      <x:c r="G21" s="14"/>
-      <x:c r="H21" s="14"/>
-      <x:c r="I21" s="14"/>
-      <x:c r="J21" s="14"/>
-      <x:c r="K21" s="14"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="14"/>
-      <x:c r="B22" s="14"/>
-      <x:c r="C22" s="15"/>
-      <x:c r="D22" s="14"/>
-      <x:c r="E22" s="14"/>
-      <x:c r="F22" s="14"/>
-      <x:c r="G22" s="14"/>
-      <x:c r="H22" s="14"/>
-      <x:c r="I22" s="14"/>
-      <x:c r="J22" s="14"/>
-      <x:c r="K22" s="14"/>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="14"/>
-      <x:c r="B23" s="14"/>
-      <x:c r="C23" s="15"/>
-      <x:c r="D23" s="14"/>
-      <x:c r="E23" s="14"/>
-      <x:c r="F23" s="14"/>
-      <x:c r="G23" s="14"/>
-      <x:c r="H23" s="14"/>
-      <x:c r="I23" s="14"/>
-      <x:c r="J23" s="14"/>
-      <x:c r="K23" s="14"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="14"/>
-      <x:c r="B24" s="14"/>
-      <x:c r="C24" s="15"/>
-      <x:c r="D24" s="14"/>
-      <x:c r="E24" s="14"/>
-      <x:c r="F24" s="14"/>
-      <x:c r="G24" s="14"/>
-      <x:c r="H24" s="14"/>
-      <x:c r="I24" s="14"/>
-      <x:c r="J24" s="14"/>
-      <x:c r="K24" s="14"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="14"/>
-      <x:c r="B25" s="14"/>
-      <x:c r="C25" s="15"/>
-      <x:c r="D25" s="14"/>
-      <x:c r="E25" s="14"/>
-      <x:c r="F25" s="14"/>
-      <x:c r="G25" s="14"/>
-      <x:c r="H25" s="14"/>
-      <x:c r="I25" s="14"/>
-      <x:c r="J25" s="14"/>
-      <x:c r="K25" s="14"/>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="14"/>
-      <x:c r="B26" s="14"/>
-      <x:c r="C26" s="15"/>
-      <x:c r="D26" s="14"/>
-      <x:c r="E26" s="14"/>
-      <x:c r="F26" s="14"/>
-      <x:c r="G26" s="14"/>
-      <x:c r="H26" s="14"/>
-      <x:c r="I26" s="14"/>
-      <x:c r="J26" s="14"/>
-      <x:c r="K26" s="14"/>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="14"/>
-      <x:c r="B27" s="14"/>
-      <x:c r="C27" s="15"/>
-      <x:c r="D27" s="14"/>
-      <x:c r="E27" s="14"/>
-      <x:c r="F27" s="14"/>
-      <x:c r="G27" s="14"/>
-      <x:c r="H27" s="14"/>
-      <x:c r="I27" s="14"/>
-      <x:c r="J27" s="14"/>
-      <x:c r="K27" s="14"/>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="14"/>
-      <x:c r="B28" s="14"/>
-      <x:c r="C28" s="15"/>
-      <x:c r="D28" s="14"/>
-      <x:c r="E28" s="14"/>
-      <x:c r="F28" s="14"/>
-      <x:c r="G28" s="14"/>
-      <x:c r="H28" s="14"/>
-      <x:c r="I28" s="14"/>
-      <x:c r="J28" s="14"/>
-      <x:c r="K28" s="14"/>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="14"/>
-      <x:c r="B29" s="14"/>
-      <x:c r="C29" s="15"/>
-      <x:c r="D29" s="14"/>
-      <x:c r="E29" s="14"/>
-      <x:c r="F29" s="14"/>
-      <x:c r="G29" s="14"/>
-      <x:c r="H29" s="14"/>
-      <x:c r="I29" s="14"/>
-      <x:c r="J29" s="14"/>
-      <x:c r="K29" s="14"/>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="14"/>
-      <x:c r="B30" s="14"/>
-      <x:c r="C30" s="15"/>
-      <x:c r="D30" s="14"/>
-      <x:c r="E30" s="14"/>
-      <x:c r="F30" s="14"/>
-      <x:c r="G30" s="14"/>
-      <x:c r="H30" s="14"/>
-      <x:c r="I30" s="14"/>
-      <x:c r="J30" s="14"/>
-      <x:c r="K30" s="14"/>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="14"/>
-      <x:c r="B31" s="14"/>
-      <x:c r="C31" s="15"/>
-      <x:c r="D31" s="14"/>
-      <x:c r="E31" s="14"/>
-      <x:c r="F31" s="14"/>
-      <x:c r="G31" s="14"/>
-      <x:c r="H31" s="14"/>
-      <x:c r="I31" s="14"/>
-      <x:c r="J31" s="14"/>
-      <x:c r="K31" s="14"/>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="14"/>
-      <x:c r="B32" s="14"/>
-      <x:c r="C32" s="15"/>
-      <x:c r="D32" s="14"/>
-      <x:c r="E32" s="14"/>
-      <x:c r="F32" s="14"/>
-      <x:c r="G32" s="14"/>
-      <x:c r="H32" s="14"/>
-      <x:c r="I32" s="14"/>
-      <x:c r="J32" s="14"/>
-      <x:c r="K32" s="14"/>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="14"/>
-      <x:c r="B33" s="14"/>
-      <x:c r="C33" s="15"/>
-      <x:c r="D33" s="14"/>
-      <x:c r="E33" s="14"/>
-      <x:c r="F33" s="14"/>
-      <x:c r="G33" s="14"/>
-      <x:c r="H33" s="14"/>
-      <x:c r="I33" s="14"/>
-      <x:c r="J33" s="14"/>
-      <x:c r="K33" s="14"/>
-    </x:row>
-  </x:sheetData>
-  <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="B4:B33">
-      <x:formula1>"原始数据,访谈,观察,测评,学生作品,照片,文件,审批,传播证明"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="I4:I33">
-      <x:formula1>"机密,内部,报送,匿名,公开"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="J4:J33">
-      <x:formula1>"计划,待授权,已采集,已核验,限制使用"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2006fe2e75484b58"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="68" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="38" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="38" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="28" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="34" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="68" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="22" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="2" t="str">
-        <x:v>真实照片证据登记</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -4079,7 +3597,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="5" t="str">
-        <x:v>只登记教师/学校真实提供的照片；不得用AI或网络图片冒充研究过程。原件与派生件分别留存。</x:v>
+        <x:v>每条结论链接到真实原件；敏感原件可受控留存，不得为了交付而复制到普通材料包。</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -4098,6 +3616,659 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="str">
+        <x:v>证据ID</x:v>
+      </x:c>
+      <x:c r="B3" s="10" t="str">
+        <x:v>类型</x:v>
+      </x:c>
+      <x:c r="C3" s="10" t="str">
+        <x:v>真实日期</x:v>
+      </x:c>
+      <x:c r="D3" s="10" t="str">
+        <x:v>是否随包</x:v>
+      </x:c>
+      <x:c r="E3" s="10" t="str">
+        <x:v>交付相对路径</x:v>
+      </x:c>
+      <x:c r="F3" s="10" t="str">
+        <x:v>SHA-256</x:v>
+      </x:c>
+      <x:c r="G3" s="10" t="str">
+        <x:v>保管责任人</x:v>
+      </x:c>
+      <x:c r="H3" s="10" t="str">
+        <x:v>受控定位</x:v>
+      </x:c>
+      <x:c r="I3" s="10" t="str">
+        <x:v>保管核验日期</x:v>
+      </x:c>
+      <x:c r="J3" s="10" t="str">
+        <x:v>对应问题</x:v>
+      </x:c>
+      <x:c r="K3" s="10" t="str">
+        <x:v>对应材料</x:v>
+      </x:c>
+      <x:c r="L3" s="10" t="str">
+        <x:v>对应结论</x:v>
+      </x:c>
+      <x:c r="M3" s="10" t="str">
+        <x:v>隐私等级</x:v>
+      </x:c>
+      <x:c r="N3" s="10" t="str">
+        <x:v>授权/核验状态</x:v>
+      </x:c>
+      <x:c r="O3" s="10" t="str">
+        <x:v>责任人</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="14"/>
+      <x:c r="B4" s="14"/>
+      <x:c r="C4" s="15"/>
+      <x:c r="D4" s="14"/>
+      <x:c r="E4" s="14"/>
+      <x:c r="F4" s="14"/>
+      <x:c r="G4" s="14"/>
+      <x:c r="H4" s="14"/>
+      <x:c r="I4" s="15"/>
+      <x:c r="J4" s="14"/>
+      <x:c r="K4" s="14"/>
+      <x:c r="L4" s="14"/>
+      <x:c r="M4" s="14"/>
+      <x:c r="N4" s="14"/>
+      <x:c r="O4" s="14"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="14"/>
+      <x:c r="B5" s="14"/>
+      <x:c r="C5" s="15"/>
+      <x:c r="D5" s="14"/>
+      <x:c r="E5" s="14"/>
+      <x:c r="F5" s="14"/>
+      <x:c r="G5" s="14"/>
+      <x:c r="H5" s="14"/>
+      <x:c r="I5" s="15"/>
+      <x:c r="J5" s="14"/>
+      <x:c r="K5" s="14"/>
+      <x:c r="L5" s="14"/>
+      <x:c r="M5" s="14"/>
+      <x:c r="N5" s="14"/>
+      <x:c r="O5" s="14"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="14"/>
+      <x:c r="B6" s="14"/>
+      <x:c r="C6" s="15"/>
+      <x:c r="D6" s="14"/>
+      <x:c r="E6" s="14"/>
+      <x:c r="F6" s="14"/>
+      <x:c r="G6" s="14"/>
+      <x:c r="H6" s="14"/>
+      <x:c r="I6" s="15"/>
+      <x:c r="J6" s="14"/>
+      <x:c r="K6" s="14"/>
+      <x:c r="L6" s="14"/>
+      <x:c r="M6" s="14"/>
+      <x:c r="N6" s="14"/>
+      <x:c r="O6" s="14"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="14"/>
+      <x:c r="B7" s="14"/>
+      <x:c r="C7" s="15"/>
+      <x:c r="D7" s="14"/>
+      <x:c r="E7" s="14"/>
+      <x:c r="F7" s="14"/>
+      <x:c r="G7" s="14"/>
+      <x:c r="H7" s="14"/>
+      <x:c r="I7" s="15"/>
+      <x:c r="J7" s="14"/>
+      <x:c r="K7" s="14"/>
+      <x:c r="L7" s="14"/>
+      <x:c r="M7" s="14"/>
+      <x:c r="N7" s="14"/>
+      <x:c r="O7" s="14"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="14"/>
+      <x:c r="B8" s="14"/>
+      <x:c r="C8" s="15"/>
+      <x:c r="D8" s="14"/>
+      <x:c r="E8" s="14"/>
+      <x:c r="F8" s="14"/>
+      <x:c r="G8" s="14"/>
+      <x:c r="H8" s="14"/>
+      <x:c r="I8" s="15"/>
+      <x:c r="J8" s="14"/>
+      <x:c r="K8" s="14"/>
+      <x:c r="L8" s="14"/>
+      <x:c r="M8" s="14"/>
+      <x:c r="N8" s="14"/>
+      <x:c r="O8" s="14"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="14"/>
+      <x:c r="B9" s="14"/>
+      <x:c r="C9" s="15"/>
+      <x:c r="D9" s="14"/>
+      <x:c r="E9" s="14"/>
+      <x:c r="F9" s="14"/>
+      <x:c r="G9" s="14"/>
+      <x:c r="H9" s="14"/>
+      <x:c r="I9" s="15"/>
+      <x:c r="J9" s="14"/>
+      <x:c r="K9" s="14"/>
+      <x:c r="L9" s="14"/>
+      <x:c r="M9" s="14"/>
+      <x:c r="N9" s="14"/>
+      <x:c r="O9" s="14"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="14"/>
+      <x:c r="B10" s="14"/>
+      <x:c r="C10" s="15"/>
+      <x:c r="D10" s="14"/>
+      <x:c r="E10" s="14"/>
+      <x:c r="F10" s="14"/>
+      <x:c r="G10" s="14"/>
+      <x:c r="H10" s="14"/>
+      <x:c r="I10" s="15"/>
+      <x:c r="J10" s="14"/>
+      <x:c r="K10" s="14"/>
+      <x:c r="L10" s="14"/>
+      <x:c r="M10" s="14"/>
+      <x:c r="N10" s="14"/>
+      <x:c r="O10" s="14"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="14"/>
+      <x:c r="B11" s="14"/>
+      <x:c r="C11" s="15"/>
+      <x:c r="D11" s="14"/>
+      <x:c r="E11" s="14"/>
+      <x:c r="F11" s="14"/>
+      <x:c r="G11" s="14"/>
+      <x:c r="H11" s="14"/>
+      <x:c r="I11" s="15"/>
+      <x:c r="J11" s="14"/>
+      <x:c r="K11" s="14"/>
+      <x:c r="L11" s="14"/>
+      <x:c r="M11" s="14"/>
+      <x:c r="N11" s="14"/>
+      <x:c r="O11" s="14"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="14"/>
+      <x:c r="B12" s="14"/>
+      <x:c r="C12" s="15"/>
+      <x:c r="D12" s="14"/>
+      <x:c r="E12" s="14"/>
+      <x:c r="F12" s="14"/>
+      <x:c r="G12" s="14"/>
+      <x:c r="H12" s="14"/>
+      <x:c r="I12" s="15"/>
+      <x:c r="J12" s="14"/>
+      <x:c r="K12" s="14"/>
+      <x:c r="L12" s="14"/>
+      <x:c r="M12" s="14"/>
+      <x:c r="N12" s="14"/>
+      <x:c r="O12" s="14"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="14"/>
+      <x:c r="B13" s="14"/>
+      <x:c r="C13" s="15"/>
+      <x:c r="D13" s="14"/>
+      <x:c r="E13" s="14"/>
+      <x:c r="F13" s="14"/>
+      <x:c r="G13" s="14"/>
+      <x:c r="H13" s="14"/>
+      <x:c r="I13" s="15"/>
+      <x:c r="J13" s="14"/>
+      <x:c r="K13" s="14"/>
+      <x:c r="L13" s="14"/>
+      <x:c r="M13" s="14"/>
+      <x:c r="N13" s="14"/>
+      <x:c r="O13" s="14"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="14"/>
+      <x:c r="B14" s="14"/>
+      <x:c r="C14" s="15"/>
+      <x:c r="D14" s="14"/>
+      <x:c r="E14" s="14"/>
+      <x:c r="F14" s="14"/>
+      <x:c r="G14" s="14"/>
+      <x:c r="H14" s="14"/>
+      <x:c r="I14" s="15"/>
+      <x:c r="J14" s="14"/>
+      <x:c r="K14" s="14"/>
+      <x:c r="L14" s="14"/>
+      <x:c r="M14" s="14"/>
+      <x:c r="N14" s="14"/>
+      <x:c r="O14" s="14"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="14"/>
+      <x:c r="B15" s="14"/>
+      <x:c r="C15" s="15"/>
+      <x:c r="D15" s="14"/>
+      <x:c r="E15" s="14"/>
+      <x:c r="F15" s="14"/>
+      <x:c r="G15" s="14"/>
+      <x:c r="H15" s="14"/>
+      <x:c r="I15" s="15"/>
+      <x:c r="J15" s="14"/>
+      <x:c r="K15" s="14"/>
+      <x:c r="L15" s="14"/>
+      <x:c r="M15" s="14"/>
+      <x:c r="N15" s="14"/>
+      <x:c r="O15" s="14"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="14"/>
+      <x:c r="B16" s="14"/>
+      <x:c r="C16" s="15"/>
+      <x:c r="D16" s="14"/>
+      <x:c r="E16" s="14"/>
+      <x:c r="F16" s="14"/>
+      <x:c r="G16" s="14"/>
+      <x:c r="H16" s="14"/>
+      <x:c r="I16" s="15"/>
+      <x:c r="J16" s="14"/>
+      <x:c r="K16" s="14"/>
+      <x:c r="L16" s="14"/>
+      <x:c r="M16" s="14"/>
+      <x:c r="N16" s="14"/>
+      <x:c r="O16" s="14"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="14"/>
+      <x:c r="B17" s="14"/>
+      <x:c r="C17" s="15"/>
+      <x:c r="D17" s="14"/>
+      <x:c r="E17" s="14"/>
+      <x:c r="F17" s="14"/>
+      <x:c r="G17" s="14"/>
+      <x:c r="H17" s="14"/>
+      <x:c r="I17" s="15"/>
+      <x:c r="J17" s="14"/>
+      <x:c r="K17" s="14"/>
+      <x:c r="L17" s="14"/>
+      <x:c r="M17" s="14"/>
+      <x:c r="N17" s="14"/>
+      <x:c r="O17" s="14"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="14"/>
+      <x:c r="B18" s="14"/>
+      <x:c r="C18" s="15"/>
+      <x:c r="D18" s="14"/>
+      <x:c r="E18" s="14"/>
+      <x:c r="F18" s="14"/>
+      <x:c r="G18" s="14"/>
+      <x:c r="H18" s="14"/>
+      <x:c r="I18" s="15"/>
+      <x:c r="J18" s="14"/>
+      <x:c r="K18" s="14"/>
+      <x:c r="L18" s="14"/>
+      <x:c r="M18" s="14"/>
+      <x:c r="N18" s="14"/>
+      <x:c r="O18" s="14"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="14"/>
+      <x:c r="B19" s="14"/>
+      <x:c r="C19" s="15"/>
+      <x:c r="D19" s="14"/>
+      <x:c r="E19" s="14"/>
+      <x:c r="F19" s="14"/>
+      <x:c r="G19" s="14"/>
+      <x:c r="H19" s="14"/>
+      <x:c r="I19" s="15"/>
+      <x:c r="J19" s="14"/>
+      <x:c r="K19" s="14"/>
+      <x:c r="L19" s="14"/>
+      <x:c r="M19" s="14"/>
+      <x:c r="N19" s="14"/>
+      <x:c r="O19" s="14"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="14"/>
+      <x:c r="B20" s="14"/>
+      <x:c r="C20" s="15"/>
+      <x:c r="D20" s="14"/>
+      <x:c r="E20" s="14"/>
+      <x:c r="F20" s="14"/>
+      <x:c r="G20" s="14"/>
+      <x:c r="H20" s="14"/>
+      <x:c r="I20" s="15"/>
+      <x:c r="J20" s="14"/>
+      <x:c r="K20" s="14"/>
+      <x:c r="L20" s="14"/>
+      <x:c r="M20" s="14"/>
+      <x:c r="N20" s="14"/>
+      <x:c r="O20" s="14"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="14"/>
+      <x:c r="B21" s="14"/>
+      <x:c r="C21" s="15"/>
+      <x:c r="D21" s="14"/>
+      <x:c r="E21" s="14"/>
+      <x:c r="F21" s="14"/>
+      <x:c r="G21" s="14"/>
+      <x:c r="H21" s="14"/>
+      <x:c r="I21" s="15"/>
+      <x:c r="J21" s="14"/>
+      <x:c r="K21" s="14"/>
+      <x:c r="L21" s="14"/>
+      <x:c r="M21" s="14"/>
+      <x:c r="N21" s="14"/>
+      <x:c r="O21" s="14"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="14"/>
+      <x:c r="B22" s="14"/>
+      <x:c r="C22" s="15"/>
+      <x:c r="D22" s="14"/>
+      <x:c r="E22" s="14"/>
+      <x:c r="F22" s="14"/>
+      <x:c r="G22" s="14"/>
+      <x:c r="H22" s="14"/>
+      <x:c r="I22" s="15"/>
+      <x:c r="J22" s="14"/>
+      <x:c r="K22" s="14"/>
+      <x:c r="L22" s="14"/>
+      <x:c r="M22" s="14"/>
+      <x:c r="N22" s="14"/>
+      <x:c r="O22" s="14"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="14"/>
+      <x:c r="B23" s="14"/>
+      <x:c r="C23" s="15"/>
+      <x:c r="D23" s="14"/>
+      <x:c r="E23" s="14"/>
+      <x:c r="F23" s="14"/>
+      <x:c r="G23" s="14"/>
+      <x:c r="H23" s="14"/>
+      <x:c r="I23" s="15"/>
+      <x:c r="J23" s="14"/>
+      <x:c r="K23" s="14"/>
+      <x:c r="L23" s="14"/>
+      <x:c r="M23" s="14"/>
+      <x:c r="N23" s="14"/>
+      <x:c r="O23" s="14"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="14"/>
+      <x:c r="B24" s="14"/>
+      <x:c r="C24" s="15"/>
+      <x:c r="D24" s="14"/>
+      <x:c r="E24" s="14"/>
+      <x:c r="F24" s="14"/>
+      <x:c r="G24" s="14"/>
+      <x:c r="H24" s="14"/>
+      <x:c r="I24" s="15"/>
+      <x:c r="J24" s="14"/>
+      <x:c r="K24" s="14"/>
+      <x:c r="L24" s="14"/>
+      <x:c r="M24" s="14"/>
+      <x:c r="N24" s="14"/>
+      <x:c r="O24" s="14"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="14"/>
+      <x:c r="B25" s="14"/>
+      <x:c r="C25" s="15"/>
+      <x:c r="D25" s="14"/>
+      <x:c r="E25" s="14"/>
+      <x:c r="F25" s="14"/>
+      <x:c r="G25" s="14"/>
+      <x:c r="H25" s="14"/>
+      <x:c r="I25" s="15"/>
+      <x:c r="J25" s="14"/>
+      <x:c r="K25" s="14"/>
+      <x:c r="L25" s="14"/>
+      <x:c r="M25" s="14"/>
+      <x:c r="N25" s="14"/>
+      <x:c r="O25" s="14"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="14"/>
+      <x:c r="B26" s="14"/>
+      <x:c r="C26" s="15"/>
+      <x:c r="D26" s="14"/>
+      <x:c r="E26" s="14"/>
+      <x:c r="F26" s="14"/>
+      <x:c r="G26" s="14"/>
+      <x:c r="H26" s="14"/>
+      <x:c r="I26" s="15"/>
+      <x:c r="J26" s="14"/>
+      <x:c r="K26" s="14"/>
+      <x:c r="L26" s="14"/>
+      <x:c r="M26" s="14"/>
+      <x:c r="N26" s="14"/>
+      <x:c r="O26" s="14"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="14"/>
+      <x:c r="B27" s="14"/>
+      <x:c r="C27" s="15"/>
+      <x:c r="D27" s="14"/>
+      <x:c r="E27" s="14"/>
+      <x:c r="F27" s="14"/>
+      <x:c r="G27" s="14"/>
+      <x:c r="H27" s="14"/>
+      <x:c r="I27" s="15"/>
+      <x:c r="J27" s="14"/>
+      <x:c r="K27" s="14"/>
+      <x:c r="L27" s="14"/>
+      <x:c r="M27" s="14"/>
+      <x:c r="N27" s="14"/>
+      <x:c r="O27" s="14"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="14"/>
+      <x:c r="B28" s="14"/>
+      <x:c r="C28" s="15"/>
+      <x:c r="D28" s="14"/>
+      <x:c r="E28" s="14"/>
+      <x:c r="F28" s="14"/>
+      <x:c r="G28" s="14"/>
+      <x:c r="H28" s="14"/>
+      <x:c r="I28" s="15"/>
+      <x:c r="J28" s="14"/>
+      <x:c r="K28" s="14"/>
+      <x:c r="L28" s="14"/>
+      <x:c r="M28" s="14"/>
+      <x:c r="N28" s="14"/>
+      <x:c r="O28" s="14"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="14"/>
+      <x:c r="B29" s="14"/>
+      <x:c r="C29" s="15"/>
+      <x:c r="D29" s="14"/>
+      <x:c r="E29" s="14"/>
+      <x:c r="F29" s="14"/>
+      <x:c r="G29" s="14"/>
+      <x:c r="H29" s="14"/>
+      <x:c r="I29" s="15"/>
+      <x:c r="J29" s="14"/>
+      <x:c r="K29" s="14"/>
+      <x:c r="L29" s="14"/>
+      <x:c r="M29" s="14"/>
+      <x:c r="N29" s="14"/>
+      <x:c r="O29" s="14"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="14"/>
+      <x:c r="B30" s="14"/>
+      <x:c r="C30" s="15"/>
+      <x:c r="D30" s="14"/>
+      <x:c r="E30" s="14"/>
+      <x:c r="F30" s="14"/>
+      <x:c r="G30" s="14"/>
+      <x:c r="H30" s="14"/>
+      <x:c r="I30" s="15"/>
+      <x:c r="J30" s="14"/>
+      <x:c r="K30" s="14"/>
+      <x:c r="L30" s="14"/>
+      <x:c r="M30" s="14"/>
+      <x:c r="N30" s="14"/>
+      <x:c r="O30" s="14"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="14"/>
+      <x:c r="B31" s="14"/>
+      <x:c r="C31" s="15"/>
+      <x:c r="D31" s="14"/>
+      <x:c r="E31" s="14"/>
+      <x:c r="F31" s="14"/>
+      <x:c r="G31" s="14"/>
+      <x:c r="H31" s="14"/>
+      <x:c r="I31" s="15"/>
+      <x:c r="J31" s="14"/>
+      <x:c r="K31" s="14"/>
+      <x:c r="L31" s="14"/>
+      <x:c r="M31" s="14"/>
+      <x:c r="N31" s="14"/>
+      <x:c r="O31" s="14"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="14"/>
+      <x:c r="B32" s="14"/>
+      <x:c r="C32" s="15"/>
+      <x:c r="D32" s="14"/>
+      <x:c r="E32" s="14"/>
+      <x:c r="F32" s="14"/>
+      <x:c r="G32" s="14"/>
+      <x:c r="H32" s="14"/>
+      <x:c r="I32" s="15"/>
+      <x:c r="J32" s="14"/>
+      <x:c r="K32" s="14"/>
+      <x:c r="L32" s="14"/>
+      <x:c r="M32" s="14"/>
+      <x:c r="N32" s="14"/>
+      <x:c r="O32" s="14"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="14"/>
+      <x:c r="B33" s="14"/>
+      <x:c r="C33" s="15"/>
+      <x:c r="D33" s="14"/>
+      <x:c r="E33" s="14"/>
+      <x:c r="F33" s="14"/>
+      <x:c r="G33" s="14"/>
+      <x:c r="H33" s="14"/>
+      <x:c r="I33" s="15"/>
+      <x:c r="J33" s="14"/>
+      <x:c r="K33" s="14"/>
+      <x:c r="L33" s="14"/>
+      <x:c r="M33" s="14"/>
+      <x:c r="N33" s="14"/>
+      <x:c r="O33" s="14"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="4">
+    <x:dataValidation type="list" sqref="B4:B33">
+      <x:formula1>"原始数据,访谈,观察,测评,学生作品,照片,文件,审批,传播证明"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D4:D33">
+      <x:formula1>"是,否"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="M4:M33">
+      <x:formula1>"机密,内部,报送,匿名,公开"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="N4:N33">
+      <x:formula1>"计划,待授权,已采集,已核验,限制使用"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart ns1:id="Ref25c6ad82e24d04"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="68" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="34" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="30" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="38" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="38" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="28" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="34" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="68" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="2" t="str">
+        <x:v>真实照片证据登记</x:v>
+      </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+      <x:c r="I1" s="2"/>
+      <x:c r="J1" s="2"/>
+      <x:c r="K1" s="2"/>
+      <x:c r="L1" s="2"/>
+      <x:c r="M1" s="2"/>
+      <x:c r="N1" s="2"/>
+      <x:c r="O1" s="2"/>
+      <x:c r="P1" s="2"/>
+      <x:c r="Q1" s="2"/>
+      <x:c r="R1" s="2"/>
+      <x:c r="S1" s="2"/>
+      <x:c r="T1" s="2"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="5" t="str">
+        <x:v>只登记教师/学校真实提供的照片；原件可随包或受控留存，报送/公开派生件必须可核验。</x:v>
+      </x:c>
+      <x:c r="B2" s="5"/>
+      <x:c r="C2" s="5"/>
+      <x:c r="D2" s="5"/>
+      <x:c r="E2" s="5"/>
+      <x:c r="F2" s="5"/>
+      <x:c r="G2" s="5"/>
+      <x:c r="H2" s="5"/>
+      <x:c r="I2" s="5"/>
+      <x:c r="J2" s="5"/>
+      <x:c r="K2" s="5"/>
+      <x:c r="L2" s="5"/>
+      <x:c r="M2" s="5"/>
+      <x:c r="N2" s="5"/>
+      <x:c r="O2" s="5"/>
+      <x:c r="P2" s="5"/>
+      <x:c r="Q2" s="5"/>
+      <x:c r="R2" s="5"/>
+      <x:c r="S2" s="5"/>
+      <x:c r="T2" s="5"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="10" t="str">
         <x:v>照片ID</x:v>
       </x:c>
       <x:c r="B3" s="10" t="str">
@@ -4119,27 +4290,42 @@
         <x:v>拍摄/来源</x:v>
       </x:c>
       <x:c r="H3" s="10" t="str">
+        <x:v>是否随包</x:v>
+      </x:c>
+      <x:c r="I3" s="10" t="str">
+        <x:v>原件相对路径</x:v>
+      </x:c>
+      <x:c r="J3" s="10" t="str">
+        <x:v>保管责任人</x:v>
+      </x:c>
+      <x:c r="K3" s="10" t="str">
+        <x:v>受控定位</x:v>
+      </x:c>
+      <x:c r="L3" s="10" t="str">
+        <x:v>保管核验日期</x:v>
+      </x:c>
+      <x:c r="M3" s="10" t="str">
         <x:v>授权状态</x:v>
       </x:c>
-      <x:c r="I3" s="10" t="str">
+      <x:c r="N3" s="10" t="str">
         <x:v>人物处理</x:v>
       </x:c>
-      <x:c r="J3" s="10" t="str">
+      <x:c r="O3" s="10" t="str">
         <x:v>图题</x:v>
       </x:c>
-      <x:c r="K3" s="10" t="str">
+      <x:c r="P3" s="10" t="str">
         <x:v>替代文本</x:v>
       </x:c>
-      <x:c r="L3" s="10" t="str">
+      <x:c r="Q3" s="10" t="str">
         <x:v>对应材料/案例</x:v>
       </x:c>
-      <x:c r="M3" s="10" t="str">
+      <x:c r="R3" s="10" t="str">
         <x:v>派生文件</x:v>
       </x:c>
-      <x:c r="N3" s="10" t="str">
+      <x:c r="S3" s="10" t="str">
         <x:v>派生SHA-256</x:v>
       </x:c>
-      <x:c r="O3" s="10" t="str">
+      <x:c r="T3" s="10" t="str">
         <x:v>图号/位置</x:v>
       </x:c>
     </x:row>
@@ -4155,10 +4341,15 @@
       <x:c r="I4" s="14"/>
       <x:c r="J4" s="14"/>
       <x:c r="K4" s="14"/>
-      <x:c r="L4" s="14"/>
+      <x:c r="L4" s="15"/>
       <x:c r="M4" s="14"/>
       <x:c r="N4" s="14"/>
       <x:c r="O4" s="14"/>
+      <x:c r="P4" s="14"/>
+      <x:c r="Q4" s="14"/>
+      <x:c r="R4" s="14"/>
+      <x:c r="S4" s="14"/>
+      <x:c r="T4" s="14"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="14"/>
@@ -4172,10 +4363,15 @@
       <x:c r="I5" s="14"/>
       <x:c r="J5" s="14"/>
       <x:c r="K5" s="14"/>
-      <x:c r="L5" s="14"/>
+      <x:c r="L5" s="15"/>
       <x:c r="M5" s="14"/>
       <x:c r="N5" s="14"/>
       <x:c r="O5" s="14"/>
+      <x:c r="P5" s="14"/>
+      <x:c r="Q5" s="14"/>
+      <x:c r="R5" s="14"/>
+      <x:c r="S5" s="14"/>
+      <x:c r="T5" s="14"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="14"/>
@@ -4189,10 +4385,15 @@
       <x:c r="I6" s="14"/>
       <x:c r="J6" s="14"/>
       <x:c r="K6" s="14"/>
-      <x:c r="L6" s="14"/>
+      <x:c r="L6" s="15"/>
       <x:c r="M6" s="14"/>
       <x:c r="N6" s="14"/>
       <x:c r="O6" s="14"/>
+      <x:c r="P6" s="14"/>
+      <x:c r="Q6" s="14"/>
+      <x:c r="R6" s="14"/>
+      <x:c r="S6" s="14"/>
+      <x:c r="T6" s="14"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="14"/>
@@ -4206,10 +4407,15 @@
       <x:c r="I7" s="14"/>
       <x:c r="J7" s="14"/>
       <x:c r="K7" s="14"/>
-      <x:c r="L7" s="14"/>
+      <x:c r="L7" s="15"/>
       <x:c r="M7" s="14"/>
       <x:c r="N7" s="14"/>
       <x:c r="O7" s="14"/>
+      <x:c r="P7" s="14"/>
+      <x:c r="Q7" s="14"/>
+      <x:c r="R7" s="14"/>
+      <x:c r="S7" s="14"/>
+      <x:c r="T7" s="14"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="14"/>
@@ -4223,10 +4429,15 @@
       <x:c r="I8" s="14"/>
       <x:c r="J8" s="14"/>
       <x:c r="K8" s="14"/>
-      <x:c r="L8" s="14"/>
+      <x:c r="L8" s="15"/>
       <x:c r="M8" s="14"/>
       <x:c r="N8" s="14"/>
       <x:c r="O8" s="14"/>
+      <x:c r="P8" s="14"/>
+      <x:c r="Q8" s="14"/>
+      <x:c r="R8" s="14"/>
+      <x:c r="S8" s="14"/>
+      <x:c r="T8" s="14"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="14"/>
@@ -4240,10 +4451,15 @@
       <x:c r="I9" s="14"/>
       <x:c r="J9" s="14"/>
       <x:c r="K9" s="14"/>
-      <x:c r="L9" s="14"/>
+      <x:c r="L9" s="15"/>
       <x:c r="M9" s="14"/>
       <x:c r="N9" s="14"/>
       <x:c r="O9" s="14"/>
+      <x:c r="P9" s="14"/>
+      <x:c r="Q9" s="14"/>
+      <x:c r="R9" s="14"/>
+      <x:c r="S9" s="14"/>
+      <x:c r="T9" s="14"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="14"/>
@@ -4257,10 +4473,15 @@
       <x:c r="I10" s="14"/>
       <x:c r="J10" s="14"/>
       <x:c r="K10" s="14"/>
-      <x:c r="L10" s="14"/>
+      <x:c r="L10" s="15"/>
       <x:c r="M10" s="14"/>
       <x:c r="N10" s="14"/>
       <x:c r="O10" s="14"/>
+      <x:c r="P10" s="14"/>
+      <x:c r="Q10" s="14"/>
+      <x:c r="R10" s="14"/>
+      <x:c r="S10" s="14"/>
+      <x:c r="T10" s="14"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="14"/>
@@ -4274,10 +4495,15 @@
       <x:c r="I11" s="14"/>
       <x:c r="J11" s="14"/>
       <x:c r="K11" s="14"/>
-      <x:c r="L11" s="14"/>
+      <x:c r="L11" s="15"/>
       <x:c r="M11" s="14"/>
       <x:c r="N11" s="14"/>
       <x:c r="O11" s="14"/>
+      <x:c r="P11" s="14"/>
+      <x:c r="Q11" s="14"/>
+      <x:c r="R11" s="14"/>
+      <x:c r="S11" s="14"/>
+      <x:c r="T11" s="14"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="14"/>
@@ -4291,10 +4517,15 @@
       <x:c r="I12" s="14"/>
       <x:c r="J12" s="14"/>
       <x:c r="K12" s="14"/>
-      <x:c r="L12" s="14"/>
+      <x:c r="L12" s="15"/>
       <x:c r="M12" s="14"/>
       <x:c r="N12" s="14"/>
       <x:c r="O12" s="14"/>
+      <x:c r="P12" s="14"/>
+      <x:c r="Q12" s="14"/>
+      <x:c r="R12" s="14"/>
+      <x:c r="S12" s="14"/>
+      <x:c r="T12" s="14"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="14"/>
@@ -4308,10 +4539,15 @@
       <x:c r="I13" s="14"/>
       <x:c r="J13" s="14"/>
       <x:c r="K13" s="14"/>
-      <x:c r="L13" s="14"/>
+      <x:c r="L13" s="15"/>
       <x:c r="M13" s="14"/>
       <x:c r="N13" s="14"/>
       <x:c r="O13" s="14"/>
+      <x:c r="P13" s="14"/>
+      <x:c r="Q13" s="14"/>
+      <x:c r="R13" s="14"/>
+      <x:c r="S13" s="14"/>
+      <x:c r="T13" s="14"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="14"/>
@@ -4325,10 +4561,15 @@
       <x:c r="I14" s="14"/>
       <x:c r="J14" s="14"/>
       <x:c r="K14" s="14"/>
-      <x:c r="L14" s="14"/>
+      <x:c r="L14" s="15"/>
       <x:c r="M14" s="14"/>
       <x:c r="N14" s="14"/>
       <x:c r="O14" s="14"/>
+      <x:c r="P14" s="14"/>
+      <x:c r="Q14" s="14"/>
+      <x:c r="R14" s="14"/>
+      <x:c r="S14" s="14"/>
+      <x:c r="T14" s="14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="14"/>
@@ -4342,10 +4583,15 @@
       <x:c r="I15" s="14"/>
       <x:c r="J15" s="14"/>
       <x:c r="K15" s="14"/>
-      <x:c r="L15" s="14"/>
+      <x:c r="L15" s="15"/>
       <x:c r="M15" s="14"/>
       <x:c r="N15" s="14"/>
       <x:c r="O15" s="14"/>
+      <x:c r="P15" s="14"/>
+      <x:c r="Q15" s="14"/>
+      <x:c r="R15" s="14"/>
+      <x:c r="S15" s="14"/>
+      <x:c r="T15" s="14"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="14"/>
@@ -4359,10 +4605,15 @@
       <x:c r="I16" s="14"/>
       <x:c r="J16" s="14"/>
       <x:c r="K16" s="14"/>
-      <x:c r="L16" s="14"/>
+      <x:c r="L16" s="15"/>
       <x:c r="M16" s="14"/>
       <x:c r="N16" s="14"/>
       <x:c r="O16" s="14"/>
+      <x:c r="P16" s="14"/>
+      <x:c r="Q16" s="14"/>
+      <x:c r="R16" s="14"/>
+      <x:c r="S16" s="14"/>
+      <x:c r="T16" s="14"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="14"/>
@@ -4376,10 +4627,15 @@
       <x:c r="I17" s="14"/>
       <x:c r="J17" s="14"/>
       <x:c r="K17" s="14"/>
-      <x:c r="L17" s="14"/>
+      <x:c r="L17" s="15"/>
       <x:c r="M17" s="14"/>
       <x:c r="N17" s="14"/>
       <x:c r="O17" s="14"/>
+      <x:c r="P17" s="14"/>
+      <x:c r="Q17" s="14"/>
+      <x:c r="R17" s="14"/>
+      <x:c r="S17" s="14"/>
+      <x:c r="T17" s="14"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="14"/>
@@ -4393,10 +4649,15 @@
       <x:c r="I18" s="14"/>
       <x:c r="J18" s="14"/>
       <x:c r="K18" s="14"/>
-      <x:c r="L18" s="14"/>
+      <x:c r="L18" s="15"/>
       <x:c r="M18" s="14"/>
       <x:c r="N18" s="14"/>
       <x:c r="O18" s="14"/>
+      <x:c r="P18" s="14"/>
+      <x:c r="Q18" s="14"/>
+      <x:c r="R18" s="14"/>
+      <x:c r="S18" s="14"/>
+      <x:c r="T18" s="14"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="14"/>
@@ -4410,10 +4671,15 @@
       <x:c r="I19" s="14"/>
       <x:c r="J19" s="14"/>
       <x:c r="K19" s="14"/>
-      <x:c r="L19" s="14"/>
+      <x:c r="L19" s="15"/>
       <x:c r="M19" s="14"/>
       <x:c r="N19" s="14"/>
       <x:c r="O19" s="14"/>
+      <x:c r="P19" s="14"/>
+      <x:c r="Q19" s="14"/>
+      <x:c r="R19" s="14"/>
+      <x:c r="S19" s="14"/>
+      <x:c r="T19" s="14"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="14"/>
@@ -4427,10 +4693,15 @@
       <x:c r="I20" s="14"/>
       <x:c r="J20" s="14"/>
       <x:c r="K20" s="14"/>
-      <x:c r="L20" s="14"/>
+      <x:c r="L20" s="15"/>
       <x:c r="M20" s="14"/>
       <x:c r="N20" s="14"/>
       <x:c r="O20" s="14"/>
+      <x:c r="P20" s="14"/>
+      <x:c r="Q20" s="14"/>
+      <x:c r="R20" s="14"/>
+      <x:c r="S20" s="14"/>
+      <x:c r="T20" s="14"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="14"/>
@@ -4444,10 +4715,15 @@
       <x:c r="I21" s="14"/>
       <x:c r="J21" s="14"/>
       <x:c r="K21" s="14"/>
-      <x:c r="L21" s="14"/>
+      <x:c r="L21" s="15"/>
       <x:c r="M21" s="14"/>
       <x:c r="N21" s="14"/>
       <x:c r="O21" s="14"/>
+      <x:c r="P21" s="14"/>
+      <x:c r="Q21" s="14"/>
+      <x:c r="R21" s="14"/>
+      <x:c r="S21" s="14"/>
+      <x:c r="T21" s="14"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="14"/>
@@ -4461,10 +4737,15 @@
       <x:c r="I22" s="14"/>
       <x:c r="J22" s="14"/>
       <x:c r="K22" s="14"/>
-      <x:c r="L22" s="14"/>
+      <x:c r="L22" s="15"/>
       <x:c r="M22" s="14"/>
       <x:c r="N22" s="14"/>
       <x:c r="O22" s="14"/>
+      <x:c r="P22" s="14"/>
+      <x:c r="Q22" s="14"/>
+      <x:c r="R22" s="14"/>
+      <x:c r="S22" s="14"/>
+      <x:c r="T22" s="14"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="14"/>
@@ -4478,10 +4759,15 @@
       <x:c r="I23" s="14"/>
       <x:c r="J23" s="14"/>
       <x:c r="K23" s="14"/>
-      <x:c r="L23" s="14"/>
+      <x:c r="L23" s="15"/>
       <x:c r="M23" s="14"/>
       <x:c r="N23" s="14"/>
       <x:c r="O23" s="14"/>
+      <x:c r="P23" s="14"/>
+      <x:c r="Q23" s="14"/>
+      <x:c r="R23" s="14"/>
+      <x:c r="S23" s="14"/>
+      <x:c r="T23" s="14"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="14"/>
@@ -4495,10 +4781,15 @@
       <x:c r="I24" s="14"/>
       <x:c r="J24" s="14"/>
       <x:c r="K24" s="14"/>
-      <x:c r="L24" s="14"/>
+      <x:c r="L24" s="15"/>
       <x:c r="M24" s="14"/>
       <x:c r="N24" s="14"/>
       <x:c r="O24" s="14"/>
+      <x:c r="P24" s="14"/>
+      <x:c r="Q24" s="14"/>
+      <x:c r="R24" s="14"/>
+      <x:c r="S24" s="14"/>
+      <x:c r="T24" s="14"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="14"/>
@@ -4512,10 +4803,15 @@
       <x:c r="I25" s="14"/>
       <x:c r="J25" s="14"/>
       <x:c r="K25" s="14"/>
-      <x:c r="L25" s="14"/>
+      <x:c r="L25" s="15"/>
       <x:c r="M25" s="14"/>
       <x:c r="N25" s="14"/>
       <x:c r="O25" s="14"/>
+      <x:c r="P25" s="14"/>
+      <x:c r="Q25" s="14"/>
+      <x:c r="R25" s="14"/>
+      <x:c r="S25" s="14"/>
+      <x:c r="T25" s="14"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="14"/>
@@ -4529,10 +4825,15 @@
       <x:c r="I26" s="14"/>
       <x:c r="J26" s="14"/>
       <x:c r="K26" s="14"/>
-      <x:c r="L26" s="14"/>
+      <x:c r="L26" s="15"/>
       <x:c r="M26" s="14"/>
       <x:c r="N26" s="14"/>
       <x:c r="O26" s="14"/>
+      <x:c r="P26" s="14"/>
+      <x:c r="Q26" s="14"/>
+      <x:c r="R26" s="14"/>
+      <x:c r="S26" s="14"/>
+      <x:c r="T26" s="14"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="14"/>
@@ -4546,10 +4847,15 @@
       <x:c r="I27" s="14"/>
       <x:c r="J27" s="14"/>
       <x:c r="K27" s="14"/>
-      <x:c r="L27" s="14"/>
+      <x:c r="L27" s="15"/>
       <x:c r="M27" s="14"/>
       <x:c r="N27" s="14"/>
       <x:c r="O27" s="14"/>
+      <x:c r="P27" s="14"/>
+      <x:c r="Q27" s="14"/>
+      <x:c r="R27" s="14"/>
+      <x:c r="S27" s="14"/>
+      <x:c r="T27" s="14"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="14"/>
@@ -4563,10 +4869,15 @@
       <x:c r="I28" s="14"/>
       <x:c r="J28" s="14"/>
       <x:c r="K28" s="14"/>
-      <x:c r="L28" s="14"/>
+      <x:c r="L28" s="15"/>
       <x:c r="M28" s="14"/>
       <x:c r="N28" s="14"/>
       <x:c r="O28" s="14"/>
+      <x:c r="P28" s="14"/>
+      <x:c r="Q28" s="14"/>
+      <x:c r="R28" s="14"/>
+      <x:c r="S28" s="14"/>
+      <x:c r="T28" s="14"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="14"/>
@@ -4580,10 +4891,15 @@
       <x:c r="I29" s="14"/>
       <x:c r="J29" s="14"/>
       <x:c r="K29" s="14"/>
-      <x:c r="L29" s="14"/>
+      <x:c r="L29" s="15"/>
       <x:c r="M29" s="14"/>
       <x:c r="N29" s="14"/>
       <x:c r="O29" s="14"/>
+      <x:c r="P29" s="14"/>
+      <x:c r="Q29" s="14"/>
+      <x:c r="R29" s="14"/>
+      <x:c r="S29" s="14"/>
+      <x:c r="T29" s="14"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="14"/>
@@ -4597,10 +4913,15 @@
       <x:c r="I30" s="14"/>
       <x:c r="J30" s="14"/>
       <x:c r="K30" s="14"/>
-      <x:c r="L30" s="14"/>
+      <x:c r="L30" s="15"/>
       <x:c r="M30" s="14"/>
       <x:c r="N30" s="14"/>
       <x:c r="O30" s="14"/>
+      <x:c r="P30" s="14"/>
+      <x:c r="Q30" s="14"/>
+      <x:c r="R30" s="14"/>
+      <x:c r="S30" s="14"/>
+      <x:c r="T30" s="14"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="14"/>
@@ -4614,10 +4935,15 @@
       <x:c r="I31" s="14"/>
       <x:c r="J31" s="14"/>
       <x:c r="K31" s="14"/>
-      <x:c r="L31" s="14"/>
+      <x:c r="L31" s="15"/>
       <x:c r="M31" s="14"/>
       <x:c r="N31" s="14"/>
       <x:c r="O31" s="14"/>
+      <x:c r="P31" s="14"/>
+      <x:c r="Q31" s="14"/>
+      <x:c r="R31" s="14"/>
+      <x:c r="S31" s="14"/>
+      <x:c r="T31" s="14"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="14"/>
@@ -4631,10 +4957,15 @@
       <x:c r="I32" s="14"/>
       <x:c r="J32" s="14"/>
       <x:c r="K32" s="14"/>
-      <x:c r="L32" s="14"/>
+      <x:c r="L32" s="15"/>
       <x:c r="M32" s="14"/>
       <x:c r="N32" s="14"/>
       <x:c r="O32" s="14"/>
+      <x:c r="P32" s="14"/>
+      <x:c r="Q32" s="14"/>
+      <x:c r="R32" s="14"/>
+      <x:c r="S32" s="14"/>
+      <x:c r="T32" s="14"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="14"/>
@@ -4648,29 +4979,37 @@
       <x:c r="I33" s="14"/>
       <x:c r="J33" s="14"/>
       <x:c r="K33" s="14"/>
-      <x:c r="L33" s="14"/>
+      <x:c r="L33" s="15"/>
       <x:c r="M33" s="14"/>
       <x:c r="N33" s="14"/>
       <x:c r="O33" s="14"/>
+      <x:c r="P33" s="14"/>
+      <x:c r="Q33" s="14"/>
+      <x:c r="R33" s="14"/>
+      <x:c r="S33" s="14"/>
+      <x:c r="T33" s="14"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="H4:H33">
+      <x:formula1>"是,否"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="M4:M33">
       <x:formula1>"计划,待取得,已取得,无需,限制,撤回"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I4:I33">
+    <x:dataValidation type="list" sqref="N4:N33">
       <x:formula1>"不适用,无人脸,背影,裁切,模糊,明确同意可识别,仅限原件"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a28b7bcf31b409b"/>
+    <x:tablePart ns1:id="R980cf8653d984886"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
@@ -5269,7 +5608,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R027a7db6c8c54380"/>
+    <x:tablePart ns1:id="R3463c0817a304664"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>